<commit_message>
Phase 2: Google Calendar integration with passing tests
</commit_message>
<xml_diff>
--- a/settlement_tracker.xlsx
+++ b/settlement_tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renilsonjr/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renilsonjr/settlement-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4157F3-C342-8F4B-A17B-69D4B9F2C40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0DD5C29-366B-4047-A865-EA682CB4B19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settlements" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="43">
   <si>
     <t>💳  SETTLEMENT PAYMENT TRACKER</t>
   </si>
@@ -163,6 +163,9 @@
   </si>
   <si>
     <t xml:space="preserve">  🟢 Green text                           →  Final payment / paid off</t>
+  </si>
+  <si>
+    <t>MACBOOK</t>
   </si>
 </sst>
 </file>
@@ -334,7 +337,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -395,6 +398,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -705,7 +711,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
@@ -719,32 +725,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
     </row>
     <row r="2" spans="1:10" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
     </row>
     <row r="3" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -2761,6 +2767,351 @@
       <c r="J65" s="11" t="s">
         <v>13</v>
       </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B67" s="3">
+        <v>1</v>
+      </c>
+      <c r="C67" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D67" s="5">
+        <v>46140</v>
+      </c>
+      <c r="E67" s="4">
+        <v>749.1</v>
+      </c>
+      <c r="F67" s="6">
+        <f t="shared" ref="F67:F76" si="24">E67-C67</f>
+        <v>674.19</v>
+      </c>
+      <c r="G67" s="7" t="str">
+        <f t="shared" ref="G67:G76" ca="1" si="25">IF(F67=0,"✅ PAID OFF",IF(TODAY()&gt;D67,"⚠️ OVERDUE","🔔 Upcoming"))</f>
+        <v>🔔 Upcoming</v>
+      </c>
+      <c r="H67" s="8">
+        <f t="shared" ref="H67:H76" si="26">D67-14</f>
+        <v>46126</v>
+      </c>
+      <c r="I67" s="8">
+        <f t="shared" ref="I67:I76" si="27">D67-7</f>
+        <v>46133</v>
+      </c>
+      <c r="J67" s="9"/>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B68" s="3">
+        <v>2</v>
+      </c>
+      <c r="C68" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D68" s="5">
+        <v>46170</v>
+      </c>
+      <c r="E68" s="4">
+        <v>674.19</v>
+      </c>
+      <c r="F68" s="6">
+        <f t="shared" si="24"/>
+        <v>599.28000000000009</v>
+      </c>
+      <c r="G68" s="7" t="str">
+        <f t="shared" ca="1" si="25"/>
+        <v>🔔 Upcoming</v>
+      </c>
+      <c r="H68" s="8">
+        <f t="shared" si="26"/>
+        <v>46156</v>
+      </c>
+      <c r="I68" s="8">
+        <f t="shared" si="27"/>
+        <v>46163</v>
+      </c>
+      <c r="J68" s="9"/>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B69" s="3">
+        <v>3</v>
+      </c>
+      <c r="C69" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D69" s="5">
+        <v>46201</v>
+      </c>
+      <c r="E69" s="4">
+        <v>599.28</v>
+      </c>
+      <c r="F69" s="6">
+        <f t="shared" si="24"/>
+        <v>524.37</v>
+      </c>
+      <c r="G69" s="7" t="str">
+        <f t="shared" ca="1" si="25"/>
+        <v>🔔 Upcoming</v>
+      </c>
+      <c r="H69" s="8">
+        <f t="shared" si="26"/>
+        <v>46187</v>
+      </c>
+      <c r="I69" s="8">
+        <f t="shared" si="27"/>
+        <v>46194</v>
+      </c>
+      <c r="J69" s="9"/>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B70" s="3">
+        <v>4</v>
+      </c>
+      <c r="C70" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D70" s="5">
+        <v>46231</v>
+      </c>
+      <c r="E70" s="4">
+        <v>524.37</v>
+      </c>
+      <c r="F70" s="6">
+        <f t="shared" si="24"/>
+        <v>449.46000000000004</v>
+      </c>
+      <c r="G70" s="7" t="str">
+        <f t="shared" ca="1" si="25"/>
+        <v>🔔 Upcoming</v>
+      </c>
+      <c r="H70" s="8">
+        <f t="shared" si="26"/>
+        <v>46217</v>
+      </c>
+      <c r="I70" s="8">
+        <f t="shared" si="27"/>
+        <v>46224</v>
+      </c>
+      <c r="J70" s="9"/>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A71" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B71" s="3">
+        <v>5</v>
+      </c>
+      <c r="C71" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D71" s="5">
+        <v>46262</v>
+      </c>
+      <c r="E71" s="4">
+        <v>449.46</v>
+      </c>
+      <c r="F71" s="6">
+        <f t="shared" si="24"/>
+        <v>374.54999999999995</v>
+      </c>
+      <c r="G71" s="7" t="str">
+        <f t="shared" ca="1" si="25"/>
+        <v>🔔 Upcoming</v>
+      </c>
+      <c r="H71" s="8">
+        <f t="shared" si="26"/>
+        <v>46248</v>
+      </c>
+      <c r="I71" s="8">
+        <f t="shared" si="27"/>
+        <v>46255</v>
+      </c>
+      <c r="J71" s="9"/>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B72" s="3">
+        <v>6</v>
+      </c>
+      <c r="C72" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D72" s="5">
+        <v>46293</v>
+      </c>
+      <c r="E72" s="4">
+        <v>374.55</v>
+      </c>
+      <c r="F72" s="6">
+        <f t="shared" si="24"/>
+        <v>299.64</v>
+      </c>
+      <c r="G72" s="7" t="str">
+        <f t="shared" ca="1" si="25"/>
+        <v>🔔 Upcoming</v>
+      </c>
+      <c r="H72" s="8">
+        <f t="shared" si="26"/>
+        <v>46279</v>
+      </c>
+      <c r="I72" s="8">
+        <f t="shared" si="27"/>
+        <v>46286</v>
+      </c>
+      <c r="J72" s="9"/>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A73" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B73" s="3">
+        <v>7</v>
+      </c>
+      <c r="C73" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D73" s="5">
+        <v>46323</v>
+      </c>
+      <c r="E73" s="4">
+        <v>299.64</v>
+      </c>
+      <c r="F73" s="6">
+        <f t="shared" ref="F73:F74" si="28">E73-C73</f>
+        <v>224.73</v>
+      </c>
+      <c r="G73" s="7" t="str">
+        <f t="shared" ref="G73:G74" ca="1" si="29">IF(F73=0,"✅ PAID OFF",IF(TODAY()&gt;D73,"⚠️ OVERDUE","🔔 Upcoming"))</f>
+        <v>🔔 Upcoming</v>
+      </c>
+      <c r="H73" s="8">
+        <f t="shared" ref="H73:H74" si="30">D73-14</f>
+        <v>46309</v>
+      </c>
+      <c r="I73" s="8">
+        <f t="shared" ref="I73:I74" si="31">D73-7</f>
+        <v>46316</v>
+      </c>
+      <c r="J73" s="9"/>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B74" s="3">
+        <v>8</v>
+      </c>
+      <c r="C74" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D74" s="5">
+        <v>46354</v>
+      </c>
+      <c r="E74" s="4">
+        <v>224.73</v>
+      </c>
+      <c r="F74" s="6">
+        <f t="shared" si="28"/>
+        <v>149.82</v>
+      </c>
+      <c r="G74" s="7" t="str">
+        <f t="shared" ca="1" si="29"/>
+        <v>🔔 Upcoming</v>
+      </c>
+      <c r="H74" s="8">
+        <f t="shared" si="30"/>
+        <v>46340</v>
+      </c>
+      <c r="I74" s="8">
+        <f t="shared" si="31"/>
+        <v>46347</v>
+      </c>
+      <c r="J74" s="9"/>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B75" s="3">
+        <v>9</v>
+      </c>
+      <c r="C75" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D75" s="5">
+        <v>46384</v>
+      </c>
+      <c r="E75" s="4">
+        <v>149.82</v>
+      </c>
+      <c r="F75" s="6">
+        <f t="shared" si="24"/>
+        <v>74.91</v>
+      </c>
+      <c r="G75" s="7" t="str">
+        <f t="shared" ca="1" si="25"/>
+        <v>🔔 Upcoming</v>
+      </c>
+      <c r="H75" s="8">
+        <f t="shared" si="26"/>
+        <v>46370</v>
+      </c>
+      <c r="I75" s="8">
+        <f t="shared" si="27"/>
+        <v>46377</v>
+      </c>
+      <c r="J75" s="9"/>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A76" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B76" s="3">
+        <v>10</v>
+      </c>
+      <c r="C76" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="D76" s="5">
+        <v>46415</v>
+      </c>
+      <c r="E76" s="4">
+        <v>74.91</v>
+      </c>
+      <c r="F76" s="10">
+        <f t="shared" si="24"/>
+        <v>0</v>
+      </c>
+      <c r="G76" s="7" t="str">
+        <f t="shared" ca="1" si="25"/>
+        <v>✅ PAID OFF</v>
+      </c>
+      <c r="H76" s="8">
+        <f t="shared" si="26"/>
+        <v>46401</v>
+      </c>
+      <c r="I76" s="8">
+        <f t="shared" si="27"/>
+        <v>46408</v>
+      </c>
+      <c r="J76" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E79" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>